<commit_message>
Initial push or update project
</commit_message>
<xml_diff>
--- a/src/data-pipline/company_fundamentals.xlsx
+++ b/src/data-pipline/company_fundamentals.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://batsalani1-my.sharepoint.com/personal/datascience_enigma-digital_ai/Documents/Desktop/market-predictor/src/data-pipline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_3B0550A0114B2CDFE54878D6425DCE3A87463846" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDB2515E-3D69-44A7-9FBC-E6BC1721AD2D}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_3B0550A0114B2CDFE54878D6425DCE3A87463846" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{432761B4-1593-482A-B453-6E97BD80D3FB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2715" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1687,7 +1688,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -1743,7 +1744,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1765,6 +1766,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2055,9 +2060,9 @@
   <dimension ref="A1:K201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
     <col min="3" max="3" width="34.140625" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="27.140625" customWidth="1"/>
     <col min="6" max="6" width="16.85546875" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" customWidth="1"/>

</xml_diff>